<commit_message>
Data Processing bestanden toegevoegd
</commit_message>
<xml_diff>
--- a/Data_Processing/systeeminformatie_windows.xlsx
+++ b/Data_Processing/systeeminformatie_windows.xlsx
@@ -416,9 +416,9 @@
   <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="51" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
@@ -426,7 +426,7 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="37" customWidth="1" min="11" max="11"/>
     <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -495,54 +495,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Unluckydodo</t>
+          <t>r1094831-VirtualBox</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AMD64</t>
+          <t>x86_64</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMD64 Family 25 Model 80 Stepping 0, AuthenticAMD</t>
+          <t>x86_64</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>2301</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>7.31</v>
+        <v>4.73</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NTFS</t>
+          <t>ext4</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>236.03</v>
+        <v>24.44</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>70-9C-D1-E9-BE-BB</t>
+          <t>08:00:27:4c:9f:e5</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>10.122.1.56</t>
+          <t>10.0.2.15</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>fd17:625c:f037:2:a00:27ff:fe4c:9fe5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>fe80::a00:27ff:fe4c:9fe5</t>
         </is>
       </c>
     </row>

</xml_diff>